<commit_message>
role-info: clean (no-numbers) Vivo/ADS worksheets
Elena's cleaned versions — answer-key numeric cells removed (vivo 35→27, ads 31→24
numeric cells), all text labels/structure preserved (sharedStrings identical).

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/frontend/public/role-info/adsWorksheet.xlsx
+++ b/frontend/public/role-info/adsWorksheet.xlsx
@@ -1,21 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10621"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10531"/>
   <workbookPr date1904="1"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/garybolton/Library/CloudStorage/Dropbox/Classes/NegotiationUTD/Mod 1 Table skills/Vivo Telecom/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/emk120030/projects/games-platform/games/vivo/frontend/public/role-info/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{634E46ED-BB3A-6A46-9A20-40AAE60AF8DA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B294C7CA-6AC2-6940-8B92-CBA186BD0D43}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4680" yWindow="600" windowWidth="19040" windowHeight="17460" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="4680" yWindow="660" windowWidth="19040" windowHeight="17360" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029" iterateDelta="1E-4"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -586,9 +586,7 @@
       </c>
       <c r="C10" s="4"/>
       <c r="D10" s="4"/>
-      <c r="E10" s="12">
-        <v>40</v>
-      </c>
+      <c r="E10" s="12"/>
       <c r="F10" s="4"/>
     </row>
     <row r="11" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -626,9 +624,7 @@
       </c>
       <c r="C14" s="4"/>
       <c r="D14" s="4"/>
-      <c r="E14" s="14">
-        <v>28</v>
-      </c>
+      <c r="E14" s="14"/>
       <c r="F14" s="4"/>
     </row>
     <row r="15" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -648,9 +644,7 @@
       </c>
       <c r="C16" s="4"/>
       <c r="D16" s="4"/>
-      <c r="E16" s="14">
-        <v>0</v>
-      </c>
+      <c r="E16" s="14"/>
       <c r="F16" s="4"/>
     </row>
     <row r="17" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -670,9 +664,7 @@
       </c>
       <c r="C18" s="4"/>
       <c r="D18" s="4"/>
-      <c r="E18" s="14">
-        <v>2</v>
-      </c>
+      <c r="E18" s="14"/>
       <c r="F18" s="4"/>
     </row>
     <row r="19" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -692,9 +684,7 @@
       </c>
       <c r="C20" s="4"/>
       <c r="D20" s="4"/>
-      <c r="E20" s="14">
-        <v>1</v>
-      </c>
+      <c r="E20" s="14"/>
       <c r="F20" s="4"/>
     </row>
     <row r="21" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -724,9 +714,9 @@
       </c>
       <c r="C23" s="4"/>
       <c r="D23" s="4"/>
-      <c r="E23" s="16">
+      <c r="E23" s="16" t="str">
         <f>IF(AND(E14="",E16="",E18="",E20=""),"",SUM(E14,E16,E18,E20))</f>
-        <v>31</v>
+        <v/>
       </c>
       <c r="F23" s="4"/>
     </row>
@@ -767,9 +757,9 @@
         <v>22</v>
       </c>
       <c r="D27" s="4"/>
-      <c r="E27" s="17">
+      <c r="E27" s="17" t="str">
         <f>IF(OR(E10="",E23=""),"",E10-E23)</f>
-        <v>9</v>
+        <v/>
       </c>
       <c r="F27" s="4"/>
     </row>

</xml_diff>